<commit_message>
looked at sensitivity analysis output
</commit_message>
<xml_diff>
--- a/Provider_Stress_Output/Provider_Stress_Results.xlsx
+++ b/Provider_Stress_Output/Provider_Stress_Results.xlsx
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -417,77 +429,77 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>scenario</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>method</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>alpha</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>lookahead_days</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>penalty</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>total_assigned</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>avg_distance_km</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>util_std_dev</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>overcap_weeks_total</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>HomecareA_avg_utilization</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>HomecareB_avg_utilization</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>HomecareC_avg_utilization</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>HomecareA_overcap_weeks</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>HomecareB_overcap_weeks</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>HomecareC_overcap_weeks</t>
         </is>

</xml_diff>

<commit_message>
change to provider stress test
</commit_message>
<xml_diff>
--- a/Provider_Stress_Output/Provider_Stress_Results.xlsx
+++ b/Provider_Stress_Output/Provider_Stress_Results.xlsx
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,77 +417,77 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>scenario</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>method</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>alpha</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>lookahead_days</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>penalty</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>total_assigned</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>avg_distance_km</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>avg_travel_hours</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
         <is>
           <t>util_std_dev</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>overcap_weeks_total</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>HomecareA_avg_utilization</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>HomecareB_avg_utilization</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>HomecareC_avg_utilization</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>HomecareA_overcap_weeks</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>HomecareB_overcap_weeks</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>HomecareC_overcap_weeks</t>
         </is>
@@ -529,7 +517,7 @@
         <v>500</v>
       </c>
       <c r="G2" t="n">
-        <v>12</v>
+        <v>0.52</v>
       </c>
       <c r="H2" t="n">
         <v>0.09</v>
@@ -580,7 +568,7 @@
         <v>500</v>
       </c>
       <c r="G3" t="n">
-        <v>6</v>
+        <v>0.26</v>
       </c>
       <c r="H3" t="n">
         <v>10.48</v>
@@ -631,7 +619,7 @@
         <v>500</v>
       </c>
       <c r="G4" t="n">
-        <v>12</v>
+        <v>0.52</v>
       </c>
       <c r="H4" t="n">
         <v>0.16</v>
@@ -682,7 +670,7 @@
         <v>500</v>
       </c>
       <c r="G5" t="n">
-        <v>12.23</v>
+        <v>0.53</v>
       </c>
       <c r="H5" t="n">
         <v>0.08</v>
@@ -733,7 +721,7 @@
         <v>500</v>
       </c>
       <c r="G6" t="n">
-        <v>11.77</v>
+        <v>0.51</v>
       </c>
       <c r="H6" t="n">
         <v>3.75</v>
@@ -784,7 +772,7 @@
         <v>500</v>
       </c>
       <c r="G7" t="n">
-        <v>6</v>
+        <v>0.26</v>
       </c>
       <c r="H7" t="n">
         <v>13.32</v>
@@ -835,7 +823,7 @@
         <v>500</v>
       </c>
       <c r="G8" t="n">
-        <v>12</v>
+        <v>0.52</v>
       </c>
       <c r="H8" t="n">
         <v>14</v>
@@ -886,7 +874,7 @@
         <v>500</v>
       </c>
       <c r="G9" t="n">
-        <v>11.77</v>
+        <v>0.51</v>
       </c>
       <c r="H9" t="n">
         <v>3.75</v>
@@ -937,7 +925,7 @@
         <v>500</v>
       </c>
       <c r="G10" t="n">
-        <v>10.85</v>
+        <v>0.47</v>
       </c>
       <c r="H10" t="n">
         <v>3.75</v>
@@ -988,7 +976,7 @@
         <v>500</v>
       </c>
       <c r="G11" t="n">
-        <v>6</v>
+        <v>0.26</v>
       </c>
       <c r="H11" t="n">
         <v>11.78</v>
@@ -1039,7 +1027,7 @@
         <v>500</v>
       </c>
       <c r="G12" t="n">
-        <v>12</v>
+        <v>0.52</v>
       </c>
       <c r="H12" t="n">
         <v>14.14</v>
@@ -1090,7 +1078,7 @@
         <v>500</v>
       </c>
       <c r="G13" t="n">
-        <v>10.62</v>
+        <v>0.46</v>
       </c>
       <c r="H13" t="n">
         <v>3.75</v>
@@ -1141,7 +1129,7 @@
         <v>500</v>
       </c>
       <c r="G14" t="n">
-        <v>14.77</v>
+        <v>0.64</v>
       </c>
       <c r="H14" t="n">
         <v>3.75</v>
@@ -1192,7 +1180,7 @@
         <v>500</v>
       </c>
       <c r="G15" t="n">
-        <v>8.31</v>
+        <v>0.36</v>
       </c>
       <c r="H15" t="n">
         <v>12.51</v>
@@ -1243,7 +1231,7 @@
         <v>500</v>
       </c>
       <c r="G16" t="n">
-        <v>12</v>
+        <v>0.52</v>
       </c>
       <c r="H16" t="n">
         <v>14.28</v>
@@ -1294,7 +1282,7 @@
         <v>500</v>
       </c>
       <c r="G17" t="n">
-        <v>14.54</v>
+        <v>0.63</v>
       </c>
       <c r="H17" t="n">
         <v>3.75</v>
@@ -1345,7 +1333,7 @@
         <v>500</v>
       </c>
       <c r="G18" t="n">
-        <v>9.23</v>
+        <v>0.4</v>
       </c>
       <c r="H18" t="n">
         <v>0.9399999999999999</v>
@@ -1396,7 +1384,7 @@
         <v>500</v>
       </c>
       <c r="G19" t="n">
-        <v>6</v>
+        <v>0.26</v>
       </c>
       <c r="H19" t="n">
         <v>3.04</v>
@@ -1447,7 +1435,7 @@
         <v>500</v>
       </c>
       <c r="G20" t="n">
-        <v>12</v>
+        <v>0.52</v>
       </c>
       <c r="H20" t="n">
         <v>14</v>
@@ -1498,7 +1486,7 @@
         <v>500</v>
       </c>
       <c r="G21" t="n">
-        <v>9.460000000000001</v>
+        <v>0.41</v>
       </c>
       <c r="H21" t="n">
         <v>0.85</v>
@@ -1549,7 +1537,7 @@
         <v>500</v>
       </c>
       <c r="G22" t="n">
-        <v>12</v>
+        <v>0.52</v>
       </c>
       <c r="H22" t="n">
         <v>0.09</v>
@@ -1600,7 +1588,7 @@
         <v>500</v>
       </c>
       <c r="G23" t="n">
-        <v>7.85</v>
+        <v>0.34</v>
       </c>
       <c r="H23" t="n">
         <v>1.88</v>
@@ -1651,7 +1639,7 @@
         <v>500</v>
       </c>
       <c r="G24" t="n">
-        <v>12</v>
+        <v>0.52</v>
       </c>
       <c r="H24" t="n">
         <v>0.16</v>
@@ -1702,7 +1690,7 @@
         <v>500</v>
       </c>
       <c r="G25" t="n">
-        <v>12.23</v>
+        <v>0.53</v>
       </c>
       <c r="H25" t="n">
         <v>0.08</v>
@@ -1753,7 +1741,7 @@
         <v>500</v>
       </c>
       <c r="G26" t="n">
-        <v>12</v>
+        <v>0.52</v>
       </c>
       <c r="H26" t="n">
         <v>0.12</v>
@@ -1804,7 +1792,7 @@
         <v>500</v>
       </c>
       <c r="G27" t="n">
-        <v>8.31</v>
+        <v>0.36</v>
       </c>
       <c r="H27" t="n">
         <v>0.87</v>
@@ -1855,7 +1843,7 @@
         <v>500</v>
       </c>
       <c r="G28" t="n">
-        <v>12</v>
+        <v>0.52</v>
       </c>
       <c r="H28" t="n">
         <v>0.16</v>
@@ -1906,7 +1894,7 @@
         <v>500</v>
       </c>
       <c r="G29" t="n">
-        <v>12.23</v>
+        <v>0.53</v>
       </c>
       <c r="H29" t="n">
         <v>0.05</v>

</xml_diff>

<commit_message>
Dashboard update and slight change to provider pressure analysis
</commit_message>
<xml_diff>
--- a/Provider_Stress_Output/Provider_Stress_Results.xlsx
+++ b/Provider_Stress_Output/Provider_Stress_Results.xlsx
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -417,77 +429,77 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>scenario</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>method</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>alpha</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>lookahead_days</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>penalty</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>total_assigned</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>avg_travel_hours</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>util_std_dev</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>overcap_weeks_total</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>HomecareA_avg_utilization</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>HomecareB_avg_utilization</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>HomecareC_avg_utilization</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>HomecareA_overcap_weeks</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>HomecareB_overcap_weeks</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>HomecareC_overcap_weeks</t>
         </is>

</xml_diff>